<commit_message>
Enrich top referral partners with published business contacts
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NMAweEWeAivDB2LaXUdWXb
</commit_message>
<xml_diff>
--- a/leads/PFD_Leads_and_Referral_Partners.xlsx
+++ b/leads/PFD_Leads_and_Referral_Partners.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Direct Investor Channels" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Referral Partners'!$A$1:$S$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Referral Partners'!$A$1:$W$69</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Events (Meet Leads)'!$A$1:$G$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Direct Investor Channels'!$A$1:$D$6</definedName>
   </definedNames>
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S69"/>
+  <dimension ref="A1:W69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -456,6 +456,10 @@
     <col width="14" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
     <col width="28" customWidth="1" min="19" max="19"/>
+    <col width="26" customWidth="1" min="20" max="20"/>
+    <col width="26" customWidth="1" min="21" max="21"/>
+    <col width="26" customWidth="1" min="22" max="22"/>
+    <col width="26" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -526,17 +530,17 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Contact name (fill in)</t>
+          <t>Contact name</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Email (fill in)</t>
+          <t>Business email (published)</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Phone (fill in)</t>
+          <t>Main phone (verify before calling)</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
@@ -552,6 +556,26 @@
       <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Contact title</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Contact source URL</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Contact confidence</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Enrichment notes</t>
         </is>
       </c>
     </row>
@@ -615,7 +639,11 @@
           <t>Yes (serves HNW clients)</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>John Samtoy</t>
+        </is>
+      </c>
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr">
@@ -625,6 +653,22 @@
       </c>
       <c r="R2" s="2" t="inlineStr"/>
       <c r="S2" s="2" t="inlineStr"/>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>International Tax Partner (Irvine)</t>
+        </is>
+      </c>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>https://hcvt.com/offices-Irvine-OC</t>
+        </is>
+      </c>
+      <c r="V2" s="2" t="inlineStr"/>
+      <c r="W2" s="2" t="inlineStr">
+        <is>
+          <t>Irvine office 18565 Jamboree Rd 4th Fl; search snippet lists Samtoy direct line 714.361.7685 and email john.samtoy@hcvt.com (individual business line; not used as main). Main office phone not found. WebFetch blocked by egress proxy. Serves HNW/family offices</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -688,7 +732,11 @@
       </c>
       <c r="N3" s="2" t="inlineStr"/>
       <c r="O3" s="2" t="inlineStr"/>
-      <c r="P3" s="2" t="inlineStr"/>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>1-800-878-4051</t>
+        </is>
+      </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -696,6 +744,14 @@
       </c>
       <c r="R3" s="2" t="inlineStr"/>
       <c r="S3" s="2" t="inlineStr"/>
+      <c r="T3" s="2" t="inlineStr"/>
+      <c r="U3" s="2" t="inlineStr"/>
+      <c r="V3" s="2" t="inlineStr"/>
+      <c r="W3" s="2" t="inlineStr">
+        <is>
+          <t>Phone from kdainc.com Newport Beach page (https://kdainc.com/service-areas/orange-county/newport-beach/cpa/); no named partner found; 800 number may be national line</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -757,9 +813,17 @@
           <t>Yes (serves HNW clients)</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>Sharon Masler</t>
+        </is>
+      </c>
       <c r="O4" s="2" t="inlineStr"/>
-      <c r="P4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>(949) 857-0404</t>
+        </is>
+      </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -767,6 +831,22 @@
       </c>
       <c r="R4" s="2" t="inlineStr"/>
       <c r="S4" s="2" t="inlineStr"/>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
+          <t>https://lantern.llc/b/masler-associates-inc-irvine/book</t>
+        </is>
+      </c>
+      <c r="V4" s="2" t="inlineStr"/>
+      <c r="W4" s="2" t="inlineStr">
+        <is>
+          <t>100 Pacifica Ste 470 Irvine; serves individuals, small biz, medical practices; phone source = lantern.llc directory; website not found</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -830,7 +910,11 @@
       </c>
       <c r="N5" s="2" t="inlineStr"/>
       <c r="O5" s="2" t="inlineStr"/>
-      <c r="P5" s="2" t="inlineStr"/>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>(714) 896-0366</t>
+        </is>
+      </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -838,6 +922,18 @@
       </c>
       <c r="R5" s="2" t="inlineStr"/>
       <c r="S5" s="2" t="inlineStr"/>
+      <c r="T5" s="2" t="inlineStr"/>
+      <c r="U5" s="2" t="inlineStr">
+        <is>
+          <t>https://lantern.llc/b/bharmal-associates-inc-irvine</t>
+        </is>
+      </c>
+      <c r="V5" s="2" t="inlineStr"/>
+      <c r="W5" s="2" t="inlineStr">
+        <is>
+          <t>18301 Von Karman Ave Unit 120 Irvine; phone from directory aggregator only; website and partners not found</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -899,7 +995,11 @@
           <t>Yes (serves HNW clients)</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>Wayne Pinnell</t>
+        </is>
+      </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr">
@@ -909,6 +1009,22 @@
       </c>
       <c r="R6" s="2" t="inlineStr"/>
       <c r="S6" s="2" t="inlineStr"/>
+      <c r="T6" s="2" t="inlineStr">
+        <is>
+          <t>Managing Partner</t>
+        </is>
+      </c>
+      <c r="U6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hwcpa.com/insights/news/haskell-white-promotions-january-2024/</t>
+        </is>
+      </c>
+      <c r="V6" s="2" t="inlineStr"/>
+      <c r="W6" s="2" t="inlineStr">
+        <is>
+          <t>Website confirmed via hwcpa.com press pages; phone not in results; 300 Spectrum Center Dr Ste 300 Irvine; Pinnell is firm managing partner not HNW-specific</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -972,7 +1088,11 @@
       </c>
       <c r="N7" s="2" t="inlineStr"/>
       <c r="O7" s="2" t="inlineStr"/>
-      <c r="P7" s="2" t="inlineStr"/>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>(949) 474-0940</t>
+        </is>
+      </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -980,6 +1100,18 @@
       </c>
       <c r="R7" s="2" t="inlineStr"/>
       <c r="S7" s="2" t="inlineStr"/>
+      <c r="T7" s="2" t="inlineStr"/>
+      <c r="U7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.klw-law.com/elite-legal-counsel-orange-county</t>
+        </is>
+      </c>
+      <c r="V7" s="2" t="inlineStr"/>
+      <c r="W7" s="2" t="inlineStr">
+        <is>
+          <t>Partner surnames Kimura, London, White (first names/titles not confirmed in results); published partner emails jkimura@/wlondon@/dwhite@klw-law.com; page targets high net worth business owners; 3 Park Plaza Irvine; phone source https://www.klw-law.com/about/</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1041,9 +1173,17 @@
           <t>Yes (serves HNW clients)</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>Darlynn Campbell Morgan</t>
+        </is>
+      </c>
       <c r="O8" s="2" t="inlineStr"/>
-      <c r="P8" s="2" t="inlineStr"/>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>(949) 260-1400</t>
+        </is>
+      </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -1051,6 +1191,22 @@
       </c>
       <c r="R8" s="2" t="inlineStr"/>
       <c r="S8" s="2" t="inlineStr"/>
+      <c r="T8" s="2" t="inlineStr">
+        <is>
+          <t>Attorney (estate planning)</t>
+        </is>
+      </c>
+      <c r="U8" s="2" t="inlineStr">
+        <is>
+          <t>https://lawyers.justia.com/lawyer/darlynn-campbell-morgan-13564</t>
+        </is>
+      </c>
+      <c r="V8" s="2" t="inlineStr"/>
+      <c r="W8" s="2" t="inlineStr">
+        <is>
+          <t>1500 Quail Ste 540 Newport Beach; phone from Justia/FindLaw listings; official site not found; title as listed generically</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1112,9 +1268,17 @@
           <t>Yes (serves HNW clients)</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>John Wong</t>
+        </is>
+      </c>
       <c r="O9" s="2" t="inlineStr"/>
-      <c r="P9" s="2" t="inlineStr"/>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>949-371-5003</t>
+        </is>
+      </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -1122,6 +1286,22 @@
       </c>
       <c r="R9" s="2" t="inlineStr"/>
       <c r="S9" s="2" t="inlineStr"/>
+      <c r="T9" s="2" t="inlineStr">
+        <is>
+          <t>Attorney (CA Bar Certified Specialist; firm lead)</t>
+        </is>
+      </c>
+      <c r="U9" s="2" t="inlineStr">
+        <is>
+          <t>https://practicefinder.newpatientsinc.com/lawyer/modern-wealth-law-irvine-ca/</t>
+        </is>
+      </c>
+      <c r="V9" s="2" t="inlineStr"/>
+      <c r="W9" s="2" t="inlineStr">
+        <is>
+          <t>Phone from directory listing not firm site; 2600 Michelson Dr Ste 950 Irvine; website not found</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1154,7 +1334,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>not confirmed</t>
+          <t>https://bcslaw.com</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1185,7 +1365,11 @@
       </c>
       <c r="N10" s="2" t="inlineStr"/>
       <c r="O10" s="2" t="inlineStr"/>
-      <c r="P10" s="2" t="inlineStr"/>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>(949) 440-3217</t>
+        </is>
+      </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -1193,6 +1377,18 @@
       </c>
       <c r="R10" s="2" t="inlineStr"/>
       <c r="S10" s="2" t="inlineStr"/>
+      <c r="T10" s="2" t="inlineStr"/>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>https://lantern.llc/b/seaton-law-group-p-c-irvine/book</t>
+        </is>
+      </c>
+      <c r="V10" s="2" t="inlineStr"/>
+      <c r="W10" s="2" t="inlineStr">
+        <is>
+          <t>15615 Alton Pkwy Irvine; website/phone from directory listing (unverified on firm site); no named principal confirmed (Barry Calvin Seaton appears on a Justia profile only)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1225,7 +1421,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>not confirmed</t>
+          <t>essaylibrown.com</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1256,7 +1452,11 @@
       </c>
       <c r="N11" s="2" t="inlineStr"/>
       <c r="O11" s="2" t="inlineStr"/>
-      <c r="P11" s="2" t="inlineStr"/>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>(949) 508-2980</t>
+        </is>
+      </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -1264,6 +1464,18 @@
       </c>
       <c r="R11" s="2" t="inlineStr"/>
       <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>https://lantern.llc/b/essayli-brown-llp-irvine/book</t>
+        </is>
+      </c>
+      <c r="V11" s="2" t="inlineStr"/>
+      <c r="W11" s="2" t="inlineStr">
+        <is>
+          <t>2211 Michelson Dr Ste 900 Irvine; phone/site from aggregator; partners not identified</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1327,7 +1539,11 @@
       </c>
       <c r="N12" s="2" t="inlineStr"/>
       <c r="O12" s="2" t="inlineStr"/>
-      <c r="P12" s="2" t="inlineStr"/>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>949-752-7722</t>
+        </is>
+      </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -1335,6 +1551,18 @@
       </c>
       <c r="R12" s="2" t="inlineStr"/>
       <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>https://business.newportbeach.com/directory/Search/attorneys-estate-planning-probate-trust-law-260995?cid=378031</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr"/>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
+          <t>Phone/address (1301 Dove St Ste 900 Newport Beach) from search summary of directories; Larry Bemis deceased per OCBA; Kenneth Hodges and Stephen Bemis listed on Justia but current titles unverified; website not found</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1396,9 +1624,17 @@
           <t>Yes (serves HNW clients)</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>James Casey</t>
+        </is>
+      </c>
       <c r="O13" s="2" t="inlineStr"/>
-      <c r="P13" s="2" t="inlineStr"/>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>(949) 706-9816</t>
+        </is>
+      </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -1406,6 +1642,22 @@
       </c>
       <c r="R13" s="2" t="inlineStr"/>
       <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr">
+        <is>
+          <t>Certified Specialist in Estate Planning, Trust &amp; Probate Law (principal)</t>
+        </is>
+      </c>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>https://lawyers.uslegal.com/attorney/the-law-office-of-james-casey-15910685/</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr"/>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t>24 Corporate Plaza Ste 200 Newport Beach; HNW estate planning plus tax controversy; website not found</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1467,9 +1719,17 @@
           <t>Yes (serves HNW clients)</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>Mary Grace Finlay</t>
+        </is>
+      </c>
       <c r="O14" s="2" t="inlineStr"/>
-      <c r="P14" s="2" t="inlineStr"/>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>(949) 509-7853</t>
+        </is>
+      </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -1477,6 +1737,22 @@
       </c>
       <c r="R14" s="2" t="inlineStr"/>
       <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr">
+        <is>
+          <t>Attorney (estate planning)</t>
+        </is>
+      </c>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>https://lawyers.justia.com/lawyer/mary-grace-finlay-19462</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr"/>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>4665 MacArthur Ct Ste 205 Newport Beach; multiple numbers found (888-896-9350; 949-269-4139); not verified which is main; website not found</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1552,6 +1828,18 @@
       </c>
       <c r="R15" s="2" t="inlineStr"/>
       <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.merceradvisors.com/?p=39264</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr"/>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>No phone or named contact found in results; Physicians Financial Advisors acquired by Mercer (fa-mag.com)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1584,7 +1872,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>not confirmed</t>
+          <t>https://rockco.com</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1623,6 +1911,18 @@
       </c>
       <c r="R16" s="2" t="inlineStr"/>
       <c r="S16" s="2" t="inlineStr"/>
+      <c r="T16" s="2" t="inlineStr"/>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.getwarmer.com/firms/rockefeller-financial-llc/offices/newport-beach-ca</t>
+        </is>
+      </c>
+      <c r="V16" s="2" t="inlineStr"/>
+      <c r="W16" s="2" t="inlineStr">
+        <is>
+          <t>Newport Beach office 800 Newport Center Dr Ste 650; no local phone found; no named partner found; NY main (212) 549-5100 not Newport</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1684,7 +1984,11 @@
           <t>Yes (serves HNW clients)</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>Greg Mech</t>
+        </is>
+      </c>
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr">
@@ -1694,6 +1998,22 @@
       </c>
       <c r="R17" s="2" t="inlineStr"/>
       <c r="S17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="inlineStr">
+        <is>
+          <t>Managing Director Newport Beach office</t>
+        </is>
+      </c>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.familywealthreport.com/article.php/US-Multi_dash_Family-Office-Creates-Head-Of-New-Office-In-Newport-Beach</t>
+        </is>
+      </c>
+      <c r="V17" s="2" t="inlineStr"/>
+      <c r="W17" s="2" t="inlineStr">
+        <is>
+          <t>HQ Boise ID; phone returned was malformed so left blank; Newport Beach office phone not found</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1755,7 +2075,11 @@
           <t>Yes (serves HNW clients)</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr"/>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>Rick Smyth</t>
+        </is>
+      </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr">
@@ -1765,6 +2089,22 @@
       </c>
       <c r="R18" s="2" t="inlineStr"/>
       <c r="S18" s="2" t="inlineStr"/>
+      <c r="T18" s="2" t="inlineStr">
+        <is>
+          <t>Founder (launched firm; formal title not confirmed)</t>
+        </is>
+      </c>
+      <c r="U18" s="2" t="inlineStr">
+        <is>
+          <t>https://altss.com/profile/aionios-capital-partners</t>
+        </is>
+      </c>
+      <c r="V18" s="2" t="inlineStr"/>
+      <c r="W18" s="2" t="inlineStr">
+        <is>
+          <t>5000 Birch St West Tower Ste 3000 Newport Beach; SEC 801-121662; no phone/website found</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1826,7 +2166,11 @@
           <t>Yes (serves HNW clients)</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>Paul Merage; Richard Merage</t>
+        </is>
+      </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr">
@@ -1836,6 +2180,22 @@
       </c>
       <c r="R19" s="2" t="inlineStr"/>
       <c r="S19" s="2" t="inlineStr"/>
+      <c r="T19" s="2" t="inlineStr">
+        <is>
+          <t>Chairman; leads single family office</t>
+        </is>
+      </c>
+      <c r="U19" s="2" t="inlineStr">
+        <is>
+          <t>https://altss.com/profile/mig-capital</t>
+        </is>
+      </c>
+      <c r="V19" s="2" t="inlineStr"/>
+      <c r="W19" s="2" t="inlineStr">
+        <is>
+          <t>Described in sources as Merage family office (may not accept outside referrals); no phone/email/website found</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1899,7 +2259,11 @@
       </c>
       <c r="N20" s="2" t="inlineStr"/>
       <c r="O20" s="2" t="inlineStr"/>
-      <c r="P20" s="2" t="inlineStr"/>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>(949) 253-7920</t>
+        </is>
+      </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -1907,6 +2271,18 @@
       </c>
       <c r="R20" s="2" t="inlineStr"/>
       <c r="S20" s="2" t="inlineStr"/>
+      <c r="T20" s="2" t="inlineStr"/>
+      <c r="U20" s="2" t="inlineStr">
+        <is>
+          <t>https://ampliz.com/company/hager-pacific-properties/82466737</t>
+        </is>
+      </c>
+      <c r="V20" s="2" t="inlineStr"/>
+      <c r="W20" s="2" t="inlineStr">
+        <is>
+          <t>4100 Newport Place Dr Ste 820 Newport Beach; phone from data aggregator; real estate firm; website/contacts not found</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1972,9 +2348,17 @@
           <t>Indirect</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr"/>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>Alexey Nechay</t>
+        </is>
+      </c>
       <c r="O21" s="2" t="inlineStr"/>
-      <c r="P21" s="2" t="inlineStr"/>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>855-955-2565</t>
+        </is>
+      </c>
       <c r="Q21" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -1982,6 +2366,22 @@
       </c>
       <c r="R21" s="2" t="inlineStr"/>
       <c r="S21" s="2" t="inlineStr"/>
+      <c r="T21" s="2" t="inlineStr">
+        <is>
+          <t>CVA CHBC (broker/appraiser)</t>
+        </is>
+      </c>
+      <c r="U21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bizbuysell.com/business-broker/alexey-nechay/nechay-advisors/41929/</t>
+        </is>
+      </c>
+      <c r="V21" s="2" t="inlineStr"/>
+      <c r="W21" s="2" t="inlineStr">
+        <is>
+          <t>Phone from BizBuySell broker listing; no firm website found</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2043,7 +2443,11 @@
           <t>Indirect</t>
         </is>
       </c>
-      <c r="N22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>David Friedman</t>
+        </is>
+      </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr">
@@ -2053,6 +2457,22 @@
       </c>
       <c r="R22" s="2" t="inlineStr"/>
       <c r="S22" s="2" t="inlineStr"/>
+      <c r="T22" s="2" t="inlineStr">
+        <is>
+          <t>President, Orange County chapter</t>
+        </is>
+      </c>
+      <c r="U22" s="2" t="inlineStr">
+        <is>
+          <t>https://tcaventuregroup.com/?p=201</t>
+        </is>
+      </c>
+      <c r="V22" s="2" t="inlineStr"/>
+      <c r="W22" s="2" t="inlineStr">
+        <is>
+          <t>Based at The Cove, Irvine; no phone/email in search results</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2114,7 +2534,11 @@
           <t>Yes (serves HNW clients)</t>
         </is>
       </c>
-      <c r="N23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>Kevin Cloward</t>
+        </is>
+      </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr">
@@ -2124,6 +2548,22 @@
       </c>
       <c r="R23" s="2" t="inlineStr"/>
       <c r="S23" s="2" t="inlineStr"/>
+      <c r="T23" s="2" t="inlineStr">
+        <is>
+          <t>Managing Partner</t>
+        </is>
+      </c>
+      <c r="U23" s="2" t="inlineStr">
+        <is>
+          <t>https://capatacpa.com/about-us-2/</t>
+        </is>
+      </c>
+      <c r="V23" s="2" t="inlineStr"/>
+      <c r="W23" s="2" t="inlineStr">
+        <is>
+          <t>HQ Laguna Niguel; other partners Sal Kureh and Manny Trelles; phone not found in results</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2185,7 +2625,11 @@
           <t>Yes (serves HNW clients)</t>
         </is>
       </c>
-      <c r="N24" s="2" t="inlineStr"/>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>Charles W. Lin</t>
+        </is>
+      </c>
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr">
@@ -2195,6 +2639,22 @@
       </c>
       <c r="R24" s="2" t="inlineStr"/>
       <c r="S24" s="2" t="inlineStr"/>
+      <c r="T24" s="2" t="inlineStr">
+        <is>
+          <t>Partner; leads Trusts and Estates practice</t>
+        </is>
+      </c>
+      <c r="U24" s="2" t="inlineStr">
+        <is>
+          <t>https://procopio.com/new-trusts-estates-leader</t>
+        </is>
+      </c>
+      <c r="V24" s="2" t="inlineStr"/>
+      <c r="W24" s="2" t="inlineStr">
+        <is>
+          <t>Serves HNW clients; OC office 100 Spectrum Center Dr Ste 520 Irvine; also Renee M. Gabbard and Jason Galaif (CPA) partners; main phone not found</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2256,7 +2716,11 @@
           <t>Yes (serves HNW clients)</t>
         </is>
       </c>
-      <c r="N25" s="2" t="inlineStr"/>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>Blaine M. Brown; Ryan W. Young</t>
+        </is>
+      </c>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr">
@@ -2266,6 +2730,22 @@
       </c>
       <c r="R25" s="2" t="inlineStr"/>
       <c r="S25" s="2" t="inlineStr"/>
+      <c r="T25" s="2" t="inlineStr">
+        <is>
+          <t>Co-founders / trial attorneys</t>
+        </is>
+      </c>
+      <c r="U25" s="2" t="inlineStr">
+        <is>
+          <t>https://lawyers.uslegal.com/attorneys/estate-planning/california/newport-beach_1</t>
+        </is>
+      </c>
+      <c r="V25" s="2" t="inlineStr"/>
+      <c r="W25" s="2" t="inlineStr">
+        <is>
+          <t>2901 W Coast Hwy #200 Newport Beach; trust and estate litigation; phone/website not found</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2327,9 +2807,17 @@
           <t>Yes (serves HNW clients)</t>
         </is>
       </c>
-      <c r="N26" s="2" t="inlineStr"/>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>Timothy J. Kay</t>
+        </is>
+      </c>
       <c r="O26" s="2" t="inlineStr"/>
-      <c r="P26" s="2" t="inlineStr"/>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>(714) 427-7000</t>
+        </is>
+      </c>
       <c r="Q26" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -2337,6 +2825,22 @@
       </c>
       <c r="R26" s="2" t="inlineStr"/>
       <c r="S26" s="2" t="inlineStr"/>
+      <c r="T26" s="2" t="inlineStr">
+        <is>
+          <t>Attorney Trusts and Estates (Costa Mesa)</t>
+        </is>
+      </c>
+      <c r="U26" s="2" t="inlineStr">
+        <is>
+          <t>https://lawyers.justia.com/lawyer/timothy-kay-1468072</t>
+        </is>
+      </c>
+      <c r="V26" s="2" t="inlineStr"/>
+      <c r="W26" s="2" t="inlineStr">
+        <is>
+          <t>600 Anton Blvd Ste 1400 Costa Mesa; also Melissa Schutz estate planning/trust admin (714) 427-7516; firm phone source via search summary</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2398,9 +2902,17 @@
           <t>Yes (serves HNW clients)</t>
         </is>
       </c>
-      <c r="N27" s="2" t="inlineStr"/>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>John Thomas Cooke</t>
+        </is>
+      </c>
       <c r="O27" s="2" t="inlineStr"/>
-      <c r="P27" s="2" t="inlineStr"/>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>949-724-3880</t>
+        </is>
+      </c>
       <c r="Q27" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -2408,6 +2920,22 @@
       </c>
       <c r="R27" s="2" t="inlineStr"/>
       <c r="S27" s="2" t="inlineStr"/>
+      <c r="T27" s="2" t="inlineStr">
+        <is>
+          <t>Founder / President / Managing Member</t>
+        </is>
+      </c>
+      <c r="U27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cookewm.com/about-us</t>
+        </is>
+      </c>
+      <c r="V27" s="2" t="inlineStr"/>
+      <c r="W27" s="2" t="inlineStr">
+        <is>
+          <t>18881 Von Karman Ave Irvine; Juliette Cooke also principal; phone from search summary of firm site</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2440,7 +2968,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>not confirmed</t>
+          <t>https://windfalladvisors.com</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -2469,9 +2997,21 @@
           <t>Yes (serves HNW clients)</t>
         </is>
       </c>
-      <c r="N28" s="2" t="inlineStr"/>
-      <c r="O28" s="2" t="inlineStr"/>
-      <c r="P28" s="2" t="inlineStr"/>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>Daniel Scott Johnson</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>info@windfalladvisors.com</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>(310) 405-5114</t>
+        </is>
+      </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -2479,6 +3019,22 @@
       </c>
       <c r="R28" s="2" t="inlineStr"/>
       <c r="S28" s="2" t="inlineStr"/>
+      <c r="T28" s="2" t="inlineStr">
+        <is>
+          <t>Founder and lead financial advisor</t>
+        </is>
+      </c>
+      <c r="U28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ocbj.com/advertorials/on-the-move/windfall-advisors-celebrates-award-win/</t>
+        </is>
+      </c>
+      <c r="V28" s="2" t="inlineStr"/>
+      <c r="W28" s="2" t="inlineStr">
+        <is>
+          <t>Contact details came from search summary without a clear source URL; address shown as 3333 Michelson Dr #300 Irvine with 310 area code (inconsistent with Newport Beach) - verify</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2540,7 +3096,11 @@
           <t>Yes (serves HNW clients)</t>
         </is>
       </c>
-      <c r="N29" s="2" t="inlineStr"/>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>Travis Allen; Mark Yates</t>
+        </is>
+      </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
       <c r="Q29" s="2" t="inlineStr">
@@ -2550,6 +3110,22 @@
       </c>
       <c r="R29" s="2" t="inlineStr"/>
       <c r="S29" s="2" t="inlineStr"/>
+      <c r="T29" s="2" t="inlineStr">
+        <is>
+          <t>CFP principals (per aggregator)</t>
+        </is>
+      </c>
+      <c r="U29" s="2" t="inlineStr">
+        <is>
+          <t>https://altss.com/profile/wealth-strategies-group</t>
+        </is>
+      </c>
+      <c r="V29" s="2" t="inlineStr"/>
+      <c r="W29" s="2" t="inlineStr">
+        <is>
+          <t>2901 W Coast Hwy Newport Beach; RIA CRD 326407; phone not found</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2613,7 +3189,11 @@
       </c>
       <c r="N30" s="2" t="inlineStr"/>
       <c r="O30" s="2" t="inlineStr"/>
-      <c r="P30" s="2" t="inlineStr"/>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>949-718-1600</t>
+        </is>
+      </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -2621,6 +3201,18 @@
       </c>
       <c r="R30" s="2" t="inlineStr"/>
       <c r="S30" s="2" t="inlineStr"/>
+      <c r="T30" s="2" t="inlineStr"/>
+      <c r="U30" s="2" t="inlineStr">
+        <is>
+          <t>https://beaconpointe.com/financial-advisors/ca/newport-beach/</t>
+        </is>
+      </c>
+      <c r="V30" s="2" t="inlineStr"/>
+      <c r="W30" s="2" t="inlineStr">
+        <is>
+          <t>24 Corporate Plaza Dr Ste 150 Newport Beach; no named principal found</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2653,7 +3245,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>not confirmed</t>
+          <t>https://www.sageviewadvisory.com</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -2684,7 +3276,11 @@
       </c>
       <c r="N31" s="2" t="inlineStr"/>
       <c r="O31" s="2" t="inlineStr"/>
-      <c r="P31" s="2" t="inlineStr"/>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>(800) 814-8742</t>
+        </is>
+      </c>
       <c r="Q31" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -2692,6 +3288,18 @@
       </c>
       <c r="R31" s="2" t="inlineStr"/>
       <c r="S31" s="2" t="inlineStr"/>
+      <c r="T31" s="2" t="inlineStr"/>
+      <c r="U31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sageviewadvisory.com/newport-beach-ca-hq</t>
+        </is>
+      </c>
+      <c r="V31" s="2" t="inlineStr"/>
+      <c r="W31" s="2" t="inlineStr">
+        <is>
+          <t>Newport Beach HQ 4000 MacArthur Blvd Ste 1050; retirement plan/wealth advisory; no named principal found</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2753,9 +3361,17 @@
           <t>Yes (serves HNW clients)</t>
         </is>
       </c>
-      <c r="N32" s="2" t="inlineStr"/>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>Zane Keller; Rick Keller</t>
+        </is>
+      </c>
       <c r="O32" s="2" t="inlineStr"/>
-      <c r="P32" s="2" t="inlineStr"/>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>714-393-0959</t>
+        </is>
+      </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -2763,6 +3379,22 @@
       </c>
       <c r="R32" s="2" t="inlineStr"/>
       <c r="S32" s="2" t="inlineStr"/>
+      <c r="T32" s="2" t="inlineStr">
+        <is>
+          <t>CEO; Chairman/Chief Economist</t>
+        </is>
+      </c>
+      <c r="U32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.businesswire.com/news/home/20250728103473/en/Introducing-Ducere-Wealth-A-Legacy-Backed-Forward-Looking-Wealth-Management-Firm</t>
+        </is>
+      </c>
+      <c r="V32" s="2" t="inlineStr"/>
+      <c r="W32" s="2" t="inlineStr">
+        <is>
+          <t>1401 Dove St Ste 630 Newport Beach; titles from press release; phone from search summary of aggregator; website not found</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2795,7 +3427,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>not confirmed</t>
+          <t>https://redmountpartners.com</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -2826,7 +3458,11 @@
       </c>
       <c r="N33" s="2" t="inlineStr"/>
       <c r="O33" s="2" t="inlineStr"/>
-      <c r="P33" s="2" t="inlineStr"/>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>949-423-3785</t>
+        </is>
+      </c>
       <c r="Q33" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -2834,6 +3470,18 @@
       </c>
       <c r="R33" s="2" t="inlineStr"/>
       <c r="S33" s="2" t="inlineStr"/>
+      <c r="T33" s="2" t="inlineStr"/>
+      <c r="U33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.getwarmer.com/firms/redmount-capital-partners-llc/offices/newport-beach-ca</t>
+        </is>
+      </c>
+      <c r="V33" s="2" t="inlineStr"/>
+      <c r="W33" s="2" t="inlineStr">
+        <is>
+          <t>23 Corporate Plaza Dr Ste 150 Newport Beach; advisors Armen Grigorian and Curtis Hollowell listed (no titles); redmountpartners.com domain appeared in results but may be a different firm (Red Mountain) - unverified</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2895,7 +3543,11 @@
           <t>Yes (serves HNW clients)</t>
         </is>
       </c>
-      <c r="N34" s="2" t="inlineStr"/>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>Benjamin Durrant; Kevin Murphy</t>
+        </is>
+      </c>
       <c r="O34" s="2" t="inlineStr"/>
       <c r="P34" s="2" t="inlineStr"/>
       <c r="Q34" s="2" t="inlineStr">
@@ -2905,6 +3557,22 @@
       </c>
       <c r="R34" s="2" t="inlineStr"/>
       <c r="S34" s="2" t="inlineStr"/>
+      <c r="T34" s="2" t="inlineStr">
+        <is>
+          <t>Founders</t>
+        </is>
+      </c>
+      <c r="U34" s="2" t="inlineStr">
+        <is>
+          <t>https://fintrx.com/firms/firm/provenio-capital-333009</t>
+        </is>
+      </c>
+      <c r="V34" s="2" t="inlineStr"/>
+      <c r="W34" s="2" t="inlineStr">
+        <is>
+          <t>SEC-registered RIA, ~76% HNWI clients, $1.6B AUM; no phone/email/website found</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2937,7 +3605,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>not confirmed</t>
+          <t>CrossRoadsBusiness.com</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2976,6 +3644,18 @@
       </c>
       <c r="R35" s="2" t="inlineStr"/>
       <c r="S35" s="2" t="inlineStr"/>
+      <c r="T35" s="2" t="inlineStr"/>
+      <c r="U35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ibba.org/state/california/</t>
+        </is>
+      </c>
+      <c r="V35" s="2" t="inlineStr"/>
+      <c r="W35" s="2" t="inlineStr">
+        <is>
+          <t>Listed at 7700 Irvine Center Dr Ste 800 Irvine (not Newport Beach); phone not shown</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3008,7 +3688,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>not confirmed</t>
+          <t>https://hardmoneylendersorangecounty.com/</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -3039,7 +3719,11 @@
       </c>
       <c r="N36" s="2" t="inlineStr"/>
       <c r="O36" s="2" t="inlineStr"/>
-      <c r="P36" s="2" t="inlineStr"/>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>714-455-3067</t>
+        </is>
+      </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -3047,6 +3731,18 @@
       </c>
       <c r="R36" s="2" t="inlineStr"/>
       <c r="S36" s="2" t="inlineStr"/>
+      <c r="T36" s="2" t="inlineStr"/>
+      <c r="U36" s="2" t="inlineStr">
+        <is>
+          <t>https://hardmoneylendersorangecounty.com/</t>
+        </is>
+      </c>
+      <c r="V36" s="2" t="inlineStr"/>
+      <c r="W36" s="2" t="inlineStr">
+        <is>
+          <t>520 Newport Center Dr Newport Beach per search summary; no named contact</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3118,6 +3814,18 @@
       </c>
       <c r="R37" s="2" t="inlineStr"/>
       <c r="S37" s="2" t="inlineStr"/>
+      <c r="T37" s="2" t="inlineStr"/>
+      <c r="U37" s="2" t="inlineStr">
+        <is>
+          <t>https://aaplonline.com/?p=12707</t>
+        </is>
+      </c>
+      <c r="V37" s="2" t="inlineStr"/>
+      <c r="W37" s="2" t="inlineStr">
+        <is>
+          <t>Private lender HQ Newport Beach, founded 2013; no phone/email/website/names found</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3179,9 +3887,17 @@
           <t>Indirect</t>
         </is>
       </c>
-      <c r="N38" s="2" t="inlineStr"/>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>Kaaren Hall</t>
+        </is>
+      </c>
       <c r="O38" s="2" t="inlineStr"/>
-      <c r="P38" s="2" t="inlineStr"/>
+      <c r="P38" s="2" t="inlineStr">
+        <is>
+          <t>866-200-1435</t>
+        </is>
+      </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -3189,6 +3905,22 @@
       </c>
       <c r="R38" s="2" t="inlineStr"/>
       <c r="S38" s="2" t="inlineStr"/>
+      <c r="T38" s="2" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="U38" s="2" t="inlineStr">
+        <is>
+          <t>https://meetup.com/orange-county-real-estate-investors-association-ocreia</t>
+        </is>
+      </c>
+      <c r="V38" s="2" t="inlineStr"/>
+      <c r="W38" s="2" t="inlineStr">
+        <is>
+          <t>Meets Wyndham 3350 Ave of the Arts Costa Mesa; association not a firm; phone source unverified</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3260,6 +3992,18 @@
       </c>
       <c r="R39" s="2" t="inlineStr"/>
       <c r="S39" s="2" t="inlineStr"/>
+      <c r="T39" s="2" t="inlineStr"/>
+      <c r="U39" s="2" t="inlineStr">
+        <is>
+          <t>https://meetup.com/orange-county-fibi</t>
+        </is>
+      </c>
+      <c r="V39" s="2" t="inlineStr"/>
+      <c r="W39" s="2" t="inlineStr">
+        <is>
+          <t>Meetup group (11k+ members) meets 1st Tuesday Irvine; no business phone/contact; networking venue not firm</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3292,7 +4036,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>not confirmed</t>
+          <t>https://gilltaxgroup.com</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -3321,7 +4065,11 @@
           <t>Yes (serves HNW clients)</t>
         </is>
       </c>
-      <c r="N40" s="2" t="inlineStr"/>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>Divya K. Gill</t>
+        </is>
+      </c>
       <c r="O40" s="2" t="inlineStr"/>
       <c r="P40" s="2" t="inlineStr"/>
       <c r="Q40" s="2" t="inlineStr">
@@ -3331,6 +4079,22 @@
       </c>
       <c r="R40" s="2" t="inlineStr"/>
       <c r="S40" s="2" t="inlineStr"/>
+      <c r="T40" s="2" t="inlineStr">
+        <is>
+          <t>Owner, CPA</t>
+        </is>
+      </c>
+      <c r="U40" s="2" t="inlineStr">
+        <is>
+          <t>https://parse.gl/brands/gilltaxgroup-com</t>
+        </is>
+      </c>
+      <c r="V40" s="2" t="inlineStr"/>
+      <c r="W40" s="2" t="inlineStr">
+        <is>
+          <t>Offices Santa Monica, Irvine, San Diego; website inferred from directory brand page; no phone found</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3402,6 +4166,14 @@
       </c>
       <c r="R41" s="2" t="inlineStr"/>
       <c r="S41" s="2" t="inlineStr"/>
+      <c r="T41" s="2" t="inlineStr"/>
+      <c r="U41" s="2" t="inlineStr"/>
+      <c r="V41" s="2" t="inlineStr"/>
+      <c r="W41" s="2" t="inlineStr">
+        <is>
+          <t>Search returned only unrelated physician results; nothing found</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3463,9 +4235,17 @@
           <t>Yes (serves HNW clients)</t>
         </is>
       </c>
-      <c r="N42" s="2" t="inlineStr"/>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>Ken Eremita</t>
+        </is>
+      </c>
       <c r="O42" s="2" t="inlineStr"/>
-      <c r="P42" s="2" t="inlineStr"/>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>323-577-9897</t>
+        </is>
+      </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -3473,6 +4253,22 @@
       </c>
       <c r="R42" s="2" t="inlineStr"/>
       <c r="S42" s="2" t="inlineStr"/>
+      <c r="T42" s="2" t="inlineStr">
+        <is>
+          <t>CPA / Owner</t>
+        </is>
+      </c>
+      <c r="U42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.whitecoatinvestor.com/partner/ken-eremita-cpa-inc/</t>
+        </is>
+      </c>
+      <c r="V42" s="2" t="inlineStr"/>
+      <c r="W42" s="2" t="inlineStr">
+        <is>
+          <t>Serves self-employed physicians; office is 25350 Magic Mountain Pkwy Ste 300 Valencia CA (LA County not OC)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3505,7 +4301,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>not confirmed</t>
+          <t>https://earnedwealth.com</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -3548,6 +4344,18 @@
       </c>
       <c r="R43" s="2" t="inlineStr"/>
       <c r="S43" s="2" t="inlineStr"/>
+      <c r="T43" s="2" t="inlineStr"/>
+      <c r="U43" s="2" t="inlineStr">
+        <is>
+          <t>https://healthcare-brew.com/stories/2023/06/27/wealth-management-platform-earned-wants-to-help-doctors-with-financial-security</t>
+        </is>
+      </c>
+      <c r="V43" s="2" t="inlineStr"/>
+      <c r="W43" s="2" t="inlineStr">
+        <is>
+          <t>NY-based wealth/tax firm for physicians and dentists; no phone/email/named principal found; not OC-specific</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3613,8 +4421,16 @@
           <t>Yes (serves HNW clients)</t>
         </is>
       </c>
-      <c r="N44" s="2" t="inlineStr"/>
-      <c r="O44" s="2" t="inlineStr"/>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>Michelle Knight</t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>info@rwawealth.com</t>
+        </is>
+      </c>
       <c r="P44" s="2" t="inlineStr"/>
       <c r="Q44" s="2" t="inlineStr">
         <is>
@@ -3623,6 +4439,22 @@
       </c>
       <c r="R44" s="2" t="inlineStr"/>
       <c r="S44" s="2" t="inlineStr"/>
+      <c r="T44" s="2" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="U44" s="2" t="inlineStr">
+        <is>
+          <t>https://rwawealth.com/rwa-wealth-partners-executive-leadership-promotions/</t>
+        </is>
+      </c>
+      <c r="V44" s="2" t="inlineStr"/>
+      <c r="W44" s="2" t="inlineStr">
+        <is>
+          <t>Boston-area firm, no OC office confirmed. Private Wealth (617) 321-2200 info@rwawealth.com; Family Office (857) 255-2100 familyoffice@rwawealth.com; also Steve Reder President Private Wealth. Phone left in notes as no single main</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3690,7 +4522,11 @@
       </c>
       <c r="N45" s="2" t="inlineStr"/>
       <c r="O45" s="2" t="inlineStr"/>
-      <c r="P45" s="2" t="inlineStr"/>
+      <c r="P45" s="2" t="inlineStr">
+        <is>
+          <t>513-588-8080</t>
+        </is>
+      </c>
       <c r="Q45" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -3698,6 +4534,18 @@
       </c>
       <c r="R45" s="2" t="inlineStr"/>
       <c r="S45" s="2" t="inlineStr"/>
+      <c r="T45" s="2" t="inlineStr"/>
+      <c r="U45" s="2" t="inlineStr">
+        <is>
+          <t>https://www.whitecoatinvestor.com/personal-choice-financial-advisors/</t>
+        </is>
+      </c>
+      <c r="V45" s="2" t="inlineStr"/>
+      <c r="W45" s="2" t="inlineStr">
+        <is>
+          <t>Cincinnati OH (4555 Lake Forest Dr Ste 650); national physician advisor not OC; no website found</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3773,6 +4621,18 @@
       </c>
       <c r="R46" s="2" t="inlineStr"/>
       <c r="S46" s="2" t="inlineStr"/>
+      <c r="T46" s="2" t="inlineStr"/>
+      <c r="U46" s="2" t="inlineStr">
+        <is>
+          <t>https://www.whitecoatinvestor.com/white-coat-planning/</t>
+        </is>
+      </c>
+      <c r="V46" s="2" t="inlineStr"/>
+      <c r="W46" s="2" t="inlineStr">
+        <is>
+          <t>Flat-fee planning for physicians, national; no phone/email/named principal found</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3834,9 +4694,17 @@
           <t>Yes (serves HNW clients)</t>
         </is>
       </c>
-      <c r="N47" s="2" t="inlineStr"/>
+      <c r="N47" s="2" t="inlineStr">
+        <is>
+          <t>John West; Kevin Winters</t>
+        </is>
+      </c>
       <c r="O47" s="2" t="inlineStr"/>
-      <c r="P47" s="2" t="inlineStr"/>
+      <c r="P47" s="2" t="inlineStr">
+        <is>
+          <t>(949) 687-2615</t>
+        </is>
+      </c>
       <c r="Q47" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -3844,6 +4712,22 @@
       </c>
       <c r="R47" s="2" t="inlineStr"/>
       <c r="S47" s="2" t="inlineStr"/>
+      <c r="T47" s="2" t="inlineStr">
+        <is>
+          <t>Managing Partner Co-Founder (each)</t>
+        </is>
+      </c>
+      <c r="U47" s="2" t="inlineStr">
+        <is>
+          <t>https://www.theadvisoros.com/firms/flatrock-wealth-partners-llc-1777</t>
+        </is>
+      </c>
+      <c r="V47" s="2" t="inlineStr"/>
+      <c r="W47" s="2" t="inlineStr">
+        <is>
+          <t>1301 Dove St Ste 910 Newport Beach; phone from aggregator; website not found</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3915,6 +4799,18 @@
       </c>
       <c r="R48" s="2" t="inlineStr"/>
       <c r="S48" s="2" t="inlineStr"/>
+      <c r="T48" s="2" t="inlineStr"/>
+      <c r="U48" s="2" t="inlineStr">
+        <is>
+          <t>https://www.getwarmer.com/firms/pacific-specialty-investment-group-llc/offices/newport-beach-ca</t>
+        </is>
+      </c>
+      <c r="V48" s="2" t="inlineStr"/>
+      <c r="W48" s="2" t="inlineStr">
+        <is>
+          <t>4100 Campus Dr Ste 100 Newport Beach; HNW portfolio mgmt; no phone/website/contact found</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3947,7 +4843,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>not confirmed</t>
+          <t>https://www.ifa.com</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -3978,7 +4874,11 @@
       </c>
       <c r="N49" s="2" t="inlineStr"/>
       <c r="O49" s="2" t="inlineStr"/>
-      <c r="P49" s="2" t="inlineStr"/>
+      <c r="P49" s="2" t="inlineStr">
+        <is>
+          <t>(888) 643-3133</t>
+        </is>
+      </c>
       <c r="Q49" s="2" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -3986,6 +4886,18 @@
       </c>
       <c r="R49" s="2" t="inlineStr"/>
       <c r="S49" s="2" t="inlineStr"/>
+      <c r="T49" s="2" t="inlineStr"/>
+      <c r="U49" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ifa.com/aboutus</t>
+        </is>
+      </c>
+      <c r="V49" s="2" t="inlineStr"/>
+      <c r="W49" s="2" t="inlineStr">
+        <is>
+          <t>19200 Von Karman Ave Ste 150 Irvine; second number (949) 502-0050 listed; phones from search summary; no named principal found</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -5440,7 +6352,7 @@
       <c r="S69" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S69"/>
+  <autoFilter ref="A1:W69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>